<commit_message>
impl: RBAC from sec context in downstream
</commit_message>
<xml_diff>
--- a/docs/01_main-plan.xlsx
+++ b/docs/01_main-plan.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\079_data\develop\guvi-crapstone\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\079_data\develop\guvi-crapstone\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B354B76-3D03-44E5-BE2F-9F2719150416}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E81A194-C991-434C-8C34-5543F7CB0CE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{E41F4596-11FA-40CC-A5EA-B7A2DAEC2B0C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="8" xr2:uid="{E41F4596-11FA-40CC-A5EA-B7A2DAEC2B0C}"/>
   </bookViews>
   <sheets>
     <sheet name="over_all" sheetId="6" r:id="rId1"/>
@@ -5384,7 +5384,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>13</v>
       </c>

</xml_diff>